<commit_message>
Add shared QA scoring and streamlined LangGraph model comparisons
Add optional execution judging, shared criteria, and consistent timing and cost reports. Instrument API and Codex runs, reduce gateway prompt overhead, and replace implicit DeepAgents tools with explicitly configured LangGraph agents. Refresh sample and five-model comparison reports.
</commit_message>
<xml_diff>
--- a/reports/mcp_rag_chat/report.xlsx
+++ b/reports/mcp_rag_chat/report.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="172">
   <si>
     <t>Request</t>
   </si>
@@ -165,13 +165,13 @@
     <t>Run ID</t>
   </si>
   <si>
-    <t>01a0d584-f630-7ae3-97ec-7a6e46e0b422</t>
+    <t>01a1143f-a8e0-77d2-9948-24d691813660</t>
   </si>
   <si>
     <t>Recording</t>
   </si>
   <si>
-    <t>Provider trace</t>
+    <t>Offline simulation</t>
   </si>
   <si>
     <t>FX reference date</t>
@@ -216,7 +216,7 @@
     <t>Pricing scope</t>
   </si>
   <si>
-    <t>Standard online token rates. Verify rates and model access before use. Cache writes with unspecified lifetime use the 5-minute rate unless an explicit cache_write rate is configured. No batch, regional, long-context, tool, or negotiated pricing adjustments are applied.</t>
+    <t>Published online token rates verified 2026-10-05. Copilot uses GitHub rates, including saved long-context tiers, before plan allowances; these are usage estimates, not subscription invoices. Cache writes with unspecified lifetime use the 5-minute rate unless an explicit cache_write rate is configured. Direct OpenAI and Anthropic entries use standard rates; no batch, regional, tool, negotiated, or unrecorded context-tier adjustments are applied. Model availability and context capacity require separate verification.</t>
   </si>
   <si>
     <t>Model</t>
@@ -252,7 +252,7 @@
     <t>Unknown</t>
   </si>
   <si>
-    <t>2026-09-18</t>
+    <t>2026-10-05</t>
   </si>
   <si>
     <t>https://developers.openai.com/api/docs/models/gpt-5.5.md</t>
@@ -291,6 +291,99 @@
     <t>Illustrative demo rates based on openai:gpt-5.6-luna; no provider billing</t>
   </si>
   <si>
+    <t>anthropic:claude-haiku-4-5</t>
+  </si>
+  <si>
+    <t>anthropic:claude-haiku-4-5-20251001</t>
+  </si>
+  <si>
+    <t>anthropic:claude-opus-5-5</t>
+  </si>
+  <si>
+    <t>anthropic:claude-sonnet-4-6</t>
+  </si>
+  <si>
+    <t>anthropic:claude-sonnet-5-5</t>
+  </si>
+  <si>
+    <t>copilot:claude-haiku-4.5</t>
+  </si>
+  <si>
+    <t>https://docs.github.com/en/copilot/reference/copilot-billing/models-and-pricing</t>
+  </si>
+  <si>
+    <t>copilot:claude-opus-5.5</t>
+  </si>
+  <si>
+    <t>copilot:claude-sonnet-4.6</t>
+  </si>
+  <si>
+    <t>copilot:claude-sonnet-5.5</t>
+  </si>
+  <si>
+    <t>copilot:gemini-3.8-flash</t>
+  </si>
+  <si>
+    <t>copilot:gpt-5.3-codex</t>
+  </si>
+  <si>
+    <t>copilot:gpt-5.4</t>
+  </si>
+  <si>
+    <t>copilot:gpt-6-astra</t>
+  </si>
+  <si>
+    <t>copilot:gpt-6-luna</t>
+  </si>
+  <si>
+    <t>copilot:gpt-6-sol</t>
+  </si>
+  <si>
+    <t>copilot:gpt-6.1-sol</t>
+  </si>
+  <si>
+    <t>openai:gpt-6-astra</t>
+  </si>
+  <si>
+    <t>https://developers.openai.com/api/docs/models/gpt-6-astra.md</t>
+  </si>
+  <si>
+    <t>openai:gpt-6-luna</t>
+  </si>
+  <si>
+    <t>https://developers.openai.com/api/docs/models/gpt-6-luna.md</t>
+  </si>
+  <si>
+    <t>openai:gpt-6-sol</t>
+  </si>
+  <si>
+    <t>https://developers.openai.com/api/docs/models/gpt-6-sol.md</t>
+  </si>
+  <si>
+    <t>openai:gpt-6.1-sol</t>
+  </si>
+  <si>
+    <t>https://developers.openai.com/api/docs/models/gpt-6.1-sol.md</t>
+  </si>
+  <si>
+    <t>copilot:gpt-5.4 [long context]</t>
+  </si>
+  <si>
+    <t>Above 272,000 input tokens</t>
+  </si>
+  <si>
+    <t>copilot:gpt-6-astra [long context]</t>
+  </si>
+  <si>
+    <t>copilot:gpt-6-luna [long context]</t>
+  </si>
+  <si>
+    <t>copilot:gpt-6-sol [long context]</t>
+  </si>
+  <si>
+    <t>copilot:gpt-6.1-sol [long context]</t>
+  </si>
+  <si>
     <t>Run total</t>
   </si>
   <si>
@@ -303,10 +396,10 @@
     <t>LLM request</t>
   </si>
   <si>
-    <t>gpt-5.6-luna</t>
-  </si>
-  <si>
-    <t>01a0d584-f64b-7011-b991-72aa8370af78</t>
+    <t>scripted-chat</t>
+  </si>
+  <si>
+    <t>01a1143f-a8e4-74b2-aace-13a61626cc36</t>
   </si>
   <si>
     <t>Input at standard rate</t>
@@ -336,17 +429,13 @@
     <t>LLM response</t>
   </si>
   <si>
-    <t>Reasoning</t>
-  </si>
-  <si>
     <t>Output</t>
   </si>
   <si>
     <t xml:space="preserve">    Output content</t>
   </si>
   <si>
-    <t>[{"id": "rs_0b5b9623b48f7896006ab5a310eee887d2b1227fc11df199d4", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqtaMRPiOUNm5naR9hyndtJ_lYeJTIXBfQ45IpHZVpTjmqhezpcv0lWPqosP4O382CqxGHGcKmKoTJQBJxeCWzx-Q18IZXZjEcZYGo7UwMJPjHOD8C2xKeQEpTYNCWAhtetfEDgI2AZslJM7Wb4wsVEn9XrUSNkAQ9dArrYi2lbX6B7-9g-9khsQTLBncYtx124oqdCA-YbgbOcgcM7L2QHvfBMRWmC-2uvznskIYGT84ek0hDYEnQ8uxDb0cSOIXT_9xlM71Fr3RGrssUNKYB6O24G10xg9B0joB62qVnRbUv-FXHIfFFfQcHyPR-vs7Gf8mzOuoghk2H3SUGHv4cfX7MgUIE104n2fM3xbD89_PJ500JvT_Ws3PG1BlS4UYnRzqaGgrdEpFvSlt4CEEHm4ZNNoeWCRg9Y5IdH0Zvf31ZiUMVnyTsGmrA90IOuQLBmilfQzR0gJUPlX56rfVpwR1Vy2lWIjToJTSo331wUbc_-VqKCaNUbs5pOkVxZlMWye6VlQ0wsIoPr5ID7gK4HPxcz8sUh4IBBbZDNcLrn3LSELvjVDgXbb_AvqGB5lrz9lUiXUrJrdmBwXQqqEOL-494NgGGbkd1hPRpV3MEWf23U4cjvYcSYaeyXprSbptVTU5UNEwroZuV4rtzl826jVIopII-x5xUEovKhAP1GcWioU_f6xXpzvHcrpcjcgdD_Pp-BmkZ4oTI7RQiXzpSU5-G47BK6AHNcaxFRGQGmFx4viv6SuwDTiCbyNXnSjYw0AOzbdwKeEfUcoIw5t_kGC77GHpYD3VQx7Av-cJXAerM_DoQvdH08anJX9ktyQCfRuXctYXo3pXecACjGcnyIh6-2i0XmDi02vRWpq3TgW89hVykl_ltGlFXPxDvg0aO6G5i9FTNVO39HdUYwo_fnIGhq4xHmnyNVqX0Qm6dn9c5JCO3IsA-_5mYFxtBp8SS7TICJk7lTsSAyotWPw00hcPGIMaEHqygcGN-0hVPyNiPNwC_ObgbNNAXMIMT2a8U7sgLhoC2eRdt-SmyhGRhNuoil1Iz0nqA8SNdZUriKkroV0x2jdSrFZ6dzs8Jxnk71ZN0zLJnAh0aAKKlz88UlPCsASsolj2de4kuLvnqpqB1ehKMqHRb6MbERT2GPt8vlyGiAtNggM72hwV7hMuQsrqqqa9TKLYiKpQ3zpKM7iynoU__6dzSZe3c_Ll9lZ2H_lJe"}, {"type": "function_call", "name": "semantic_search_wikipedia", "arguments": "{\"query\":\"How has the Australian raven adapted to urban environments, including diet, nesting, behavior, and relationship with humans?\"}", "call_id": "call_omyI4RaihUWfWh02kANPplWc", "id": "fc_0b5b9623b48f7896006ab5a3112ea087d2a8d88b7d746d318c", "index": 1}]
-{"name": "semantic_search_wikipedia", "args": {"query": "How has the Australian raven adapted to urban environments, including diet, nesting, behavior, and relationship with humans?"}, "id": "call_omyI4RaihUWfWh02kANPplWc", "type": "tool_call"}</t>
+    <t>{"name": "semantic_search_wikipedia", "args": {"query": "How has the Australian raven adapted to urban environments?"}, "id": "wiki-mcp-search-1", "type": "tool_call"}</t>
   </si>
   <si>
     <t>Call total</t>
@@ -358,25 +447,25 @@
     <t>Tool · semantic_search_wikipedia</t>
   </si>
   <si>
-    <t>01a0d584-fcb1-7b41-bfc5-b3b9b426f069</t>
+    <t>01a1143f-a967-7930-acdb-c896fcf80e62</t>
   </si>
   <si>
     <t xml:space="preserve">    Arguments</t>
   </si>
   <si>
-    <t>{'query': 'How has the Australian raven adapted to urban environments, including diet, nesting, behavior, and relationship with humans?'}</t>
+    <t>{'query': 'How has the Australian raven adapted to urban environments?'}</t>
   </si>
   <si>
     <t xml:space="preserve">    Result</t>
   </si>
   <si>
-    <t>[{"type": "text", "text": "{\"passages\": [{\"id\": \"passage-00016828\", \"text\": \"1827, its species name highlighting its similarity with the carrion crow ( c. corone ). two subspecies are recognised, which differ slightly in calls and are quite divergent genetically. the preferred habitat is open woodland and transitional zones. it has adapted well to urban environments and is a common city bird in sydney, canberra and perth. an omnivorous and opportunistic feeder, it eats a wide variety of plant and animal material, as well as food waste from urban areas. in eastern australia its range is strongly correlated with the presence of sheep, and it has been blamed for killing lambs. however, this is very rare, and the raven most often scavenges for afterbirth and stillborn animals as well as newborn lamb faeces. the australian raven is territorial, with pairs generally bonding for life. breeding takes place between july and september, with almost no variation across its range. the nest is a bowl @ - @ shaped structure of sticks sited high in a tree, or occasionally in a man @ - @ made structure such as a windmill or other building. = =\", \"source\": \"https://huggingface.co/datasets/Salesforce/wikitext/tree/b08601e04326c79dfdd32d625aee71d232d685c3/wikitext-103-raw-v1\", \"token_start\": 188, \"token_end\": 408, \"license\": \"CC-BY-SA-3.0\", \"title\": \"Australian raven\", \"source_row\": 49964, \"cosine_distance\": 0.21683210134506226}, {\"id\": \"passage-00016845\", \"text\": \"distinguishing australian corvids has hampered understanding of seasonal movements. the australian raven is thought to be largely sedentary, with most movement of over 16 km ( 9 @. @ 9 mi ) due to flocks of non @ - @ breeding subadult birds. juvenile birds leave their parents and join flocks when they are four or five months old. smaller flocks of 8 \\u2013 30 birds stay within an area of around 260 square kilometres, while larger flocks of up to 300 birds may travel hundreds of kilometres seeking food. a single breeding pair and their brood can occupy a territory of up to around 120 hectares ( 300 acres ) and remains there year @ - @ round, though groups of ravens may enter this area to forage. australian ravens will defend their territory by chasing, dive @ - @ bombing and occasionally striking the backs of birds of prey, foxes or even people. they generally mate for life, though occasionally one male has been found to be mated with two females in adjacent territories. if the female dies, the male australian raven maintains the territory and finds another mate, while\", \"source\": \"https://huggingface.co/datasets/Salesforce/wikitext/tree/b08601e04326c79dfdd32d625aee71d232d685c3/wikitext-103-raw-v1\", \"token_start\": 3384, \"source_row\": 49964, \"license\": \"CC-BY-SA-3.0\", \"token_end\": 3604, \"title\": \"Australian raven\", \"cosine_distance\": 0.3009307384490967}, {\"id\": \"passage-00016844\", \"text\": \"areas. similarly, in inland australia it can share range with the little crow, as the two do not appear to compete. however, the ranges of similar @ - @ sized forest raven and torresian crow only narrowly overlap with the australian raven as all three compete with each other. in central and western regions, australian ravens and torresian crows vye for the scattered uncommon trees and outcrops, and only one or the other are found there. it co @ - @ occurs with the forest raven in northeastern new south wales from port stephens northwards. the australian raven has adapted very well to human habitation in some cities and is the most common corvid in canberra, sydney and perth ; in melbourne and adelaide it is replaced by the little raven, and by the torresian crow in brisbane. its large range, abundance and increasing population mean it is classified as least concern on the iucn red list. = = behaviour = = difficulties in distinguishing australian corvids has hampered understanding of seasonal movements. the australian raven is thought to be largely sedentary, with most movement of over 16 km\", \"token_start\": 3196, \"source\": \"https://huggingface.co/datasets/Salesforce/wikitext/tree/b08601e04326c79dfdd32d625aee71d232d685c3/wikitext-103-raw-v1\", \"token_end\": 3416, \"title\": \"Australian raven\", \"license\": \"CC-BY-SA-3.0\", \"source_row\": 49964, \"cosine_distance\": 0.3018089532852173}, {\"id\": \"passage-00016850\", \"text\": \"or restaurants, abattoirs, piggeries and farmyards. in one isolated study, they were observed feeding on nectar from eucalypt flowers. australian ravens sometimes forage in mixed @ - @ species flocks with any of the other four species of australian corvids. sometimes they are aggressive with little ravens if both are at a food source and drive them off, though not if the smaller species greatly outnumbers the larger. = = = breeding = = = australian ravens begin breeding once they are three years old. breeding season is from july to september, with no substantial difference in timing across its range around the country despite it inhabiting a range of diverse climates and habitats across 19 degrees of latitude. rowley has pointed out this is unusual for a bird species with a wide range and has postulated that breeding is initiated by day length. rarely, breeding can take place in may, june or october. australian ravens generally nest in tall trees, never near to the ground as some species do. the nest also functions as a lookout post and so tall or emergent\", \"title\": \"Australian raven\", \"source\": \"https://huggingface.co/datasets/Salesforce/wikitext/tree/b08601e04326c79dfdd32d625aee71d232d685c3/wikitext-103-raw-v1\", \"license\": \"CC-BY-SA-3.0\", \"token_start\": 4324, \"source_row\": 49964, \"token_end\": 4544, \"cosine_distance\": 0.3207911252975464}], \"note\": \"Nearest passages are candidates, not proof of relevance; abstain if they do not answer the question.\"}", "id": "lc_e622d6f8-26e5-46d7-986b-e6ae1ae3c69d"}]</t>
+    <t>[{"type": "text", "text": "{\"passages\": [{\"id\": \"passage-00016844\", \"text\": \"areas. similarly, in inland australia it can share range with the little crow, as the two do not appear to compete. however, the ranges of similar @ - @ sized forest raven and torresian crow only narrowly overlap with the australian raven as all three compete with each other. in central and western regions, australian ravens and torresian crows vye for the scattered uncommon trees and outcrops, and only one or the other are found there. it co @ - @ occurs with the forest raven in northeastern new south wales from port stephens northwards. the australian raven has adapted very well to human habitation in some cities and is the most common corvid in canberra, sydney and perth ; in melbourne and adelaide it is replaced by the little raven, and by the torresian crow in brisbane. its large range, abundance and increasing population mean it is classified as least concern on the iucn red list. = = behaviour = = difficulties in distinguishing australian corvids has hampered understanding of seasonal movements. the australian raven is thought to be largely sedentary, with most movement of over 16 km\", \"source\": \"https://huggingface.co/datasets/Salesforce/wikitext/tree/b08601e04326c79dfdd32d625aee71d232d685c3/wikitext-103-raw-v1\", \"token_start\": 3196, \"title\": \"Australian raven\", \"source_row\": 49964, \"license\": \"CC-BY-SA-3.0\", \"token_end\": 3416, \"cosine_distance\": 0.29966193437576294}, {\"id\": \"passage-00016828\", \"text\": \"1827, its species name highlighting its similarity with the carrion crow ( c. corone ). two subspecies are recognised, which differ slightly in calls and are quite divergent genetically. the preferred habitat is open woodland and transitional zones. it has adapted well to urban environments and is a common city bird in sydney, canberra and perth. an omnivorous and opportunistic feeder, it eats a wide variety of plant and animal material, as well as food waste from urban areas. in eastern australia its range is strongly correlated with the presence of sheep, and it has been blamed for killing lambs. however, this is very rare, and the raven most often scavenges for afterbirth and stillborn animals as well as newborn lamb faeces. the australian raven is territorial, with pairs generally bonding for life. breeding takes place between july and september, with almost no variation across its range. the nest is a bowl @ - @ shaped structure of sticks sited high in a tree, or occasionally in a man @ - @ made structure such as a windmill or other building. = =\", \"source_row\": 49964, \"token_start\": 188, \"license\": \"CC-BY-SA-3.0\", \"title\": \"Australian raven\", \"token_end\": 408, \"source\": \"https://huggingface.co/datasets/Salesforce/wikitext/tree/b08601e04326c79dfdd32d625aee71d232d685c3/wikitext-103-raw-v1\", \"cosine_distance\": 0.3006012439727783}, {\"id\": \"passage-00016843\", \"text\": \". it is rare in the australian alps, being replaced there by the little raven. it occurs across victoria and eastern south australia, through the eyre peninsula and nullarbor plain into western australia, across the state north to the wooramel river. it is found on some offshore islands such as rottnest island and kangaroo island. it is a rare vagrant to lord howe island. the australian raven can be found in a wide range of natural and modified habitats. it requires available water and trees ( or buildings ) to roost in or perch on. preferred habitats include eucalypt @ - @ dominated sclerophyll forest, and farmland adjacent to trees. it is also found in heath and mangroves. in areas where it occurs with the little raven, namely over much of central new south wales, victoria and into south australia, the australian raven is restricted to more forested areas while the latter species prefers more open areas. similarly, in inland australia it can share range with the little crow, as the two do not appear to compete. however, the ranges of similar @\", \"license\": \"CC-BY-SA-3.0\", \"title\": \"Australian raven\", \"source\": \"https://huggingface.co/datasets/Salesforce/wikitext/tree/b08601e04326c79dfdd32d625aee71d232d685c3/wikitext-103-raw-v1\", \"source_row\": 49964, \"token_start\": 3008, \"token_end\": 3228, \"cosine_distance\": 0.31825459003448486}, {\"id\": \"passage-00016845\", \"text\": \"distinguishing australian corvids has hampered understanding of seasonal movements. the australian raven is thought to be largely sedentary, with most movement of over 16 km ( 9 @. @ 9 mi ) due to flocks of non @ - @ breeding subadult birds. juvenile birds leave their parents and join flocks when they are four or five months old. smaller flocks of 8 \\u2013 30 birds stay within an area of around 260 square kilometres, while larger flocks of up to 300 birds may travel hundreds of kilometres seeking food. a single breeding pair and their brood can occupy a territory of up to around 120 hectares ( 300 acres ) and remains there year @ - @ round, though groups of ravens may enter this area to forage. australian ravens will defend their territory by chasing, dive @ - @ bombing and occasionally striking the backs of birds of prey, foxes or even people. they generally mate for life, though occasionally one male has been found to be mated with two females in adjacent territories. if the female dies, the male australian raven maintains the territory and finds another mate, while\", \"title\": \"Australian raven\", \"token_start\": 3384, \"token_end\": 3604, \"license\": \"CC-BY-SA-3.0\", \"source\": \"https://huggingface.co/datasets/Salesforce/wikitext/tree/b08601e04326c79dfdd32d625aee71d232d685c3/wikitext-103-raw-v1\", \"source_row\": 49964, \"cosine_distance\": 0.343753457069397}], \"note\": \"Nearest passages are candidates, not proof of relevance; abstain if they do not answer the question.\"}", "id": "lc_c7c58dc1-3f4e-47c3-9e8a-117ea4f43443"}]</t>
   </si>
   <si>
     <t>R2</t>
   </si>
   <si>
-    <t>01a0d585-0190-7e52-b657-fa442e1310c6</t>
+    <t>01a1143f-aaa2-76c3-807c-e7e3e39b0a0b</t>
   </si>
   <si>
     <t>Conversation history · cache read</t>
@@ -385,7 +474,7 @@
     <t xml:space="preserve">    Tool result</t>
   </si>
   <si>
-    <t>[{"type": "text", "text": "The Australian raven has adapted to cities in several ways:\n\n- **Flexible diet:** It is an opportunistic omnivore, eating plants, animals, carrion, and human food waste\u2014resources readily available in urban areas. [passage-00016828]\n- **Use of built structures:** Although it normally nests high in trees, it sometimes builds nests on man-made structures such as windmills and buildings. [passage-00016828]\n- **Urban tolerance:** It has adapted particularly well to human habitation and is a common city bird in Sydney, Canberra, and Perth. [passage-00016844]\n- **Territorial behavior remains important:** Even in urban settings, breeding pairs maintain territories and defend them from threats. [passage-00016845]\n\nOverall, its adaptability comes mainly from a broad diet, willingness to exploit human structures and waste, and the ability to persist in modified habitats.", "phase": "final_answer", "index": 0, "id": "msg_0b5b9623b48f7896006ab5a313b5b087d290a30d9a20719e2f"}]</t>
+    <t>The MCP search completed. Inspect the semantic_search_wikipedia result for retrieved passages and source IDs. This scripted response demonstrates retrieval and accounting, not answer synthesis.</t>
   </si>
   <si>
     <t>wikipedia_mcp_agent</t>
@@ -400,46 +489,37 @@
     <t>Subtree total</t>
   </si>
   <si>
-    <t xml:space="preserve">    PatchToolCallsMiddleware.before_agent</t>
-  </si>
-  <si>
-    <t>Check message history and repair missing tool responses before the agent starts.</t>
-  </si>
-  <si>
-    <t>01a0d584-f637-79f3-80ee-ab810e51617e</t>
+    <t xml:space="preserve">    model</t>
+  </si>
+  <si>
+    <t>Prepare the current conversation, run model middleware, and invoke the chat model.</t>
+  </si>
+  <si>
+    <t>01a1143f-a8e3-7263-9603-1d03839b7600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        SimulatedModel</t>
+  </si>
+  <si>
+    <t>model</t>
+  </si>
+  <si>
+    <t>Reach the local Wikipedia index through MCP.</t>
+  </si>
+  <si>
+    <t>Own call</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    tools</t>
+  </si>
+  <si>
+    <t>Execute tool calls requested by the preceding model response and return their observations.</t>
+  </si>
+  <si>
+    <t>01a1143f-a966-7320-822f-61e3c0546c12</t>
   </si>
   <si>
     <t>No model charge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    model</t>
-  </si>
-  <si>
-    <t>Prepare the current conversation, run model middleware, and invoke the chat model.</t>
-  </si>
-  <si>
-    <t>01a0d584-f63b-7933-8159-45b51cb1ab48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">        ChatOpenAI</t>
-  </si>
-  <si>
-    <t>model</t>
-  </si>
-  <si>
-    <t>Generate the next assistant message or tool request from the current conversation.</t>
-  </si>
-  <si>
-    <t>Own call</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    tools</t>
-  </si>
-  <si>
-    <t>Execute tool calls requested by the preceding model response and return their observations.</t>
-  </si>
-  <si>
-    <t>01a0d584-fcb0-74e3-bbf2-0549496496e7</t>
   </si>
   <si>
     <t xml:space="preserve">        semantic_search_wikipedia</t>
@@ -452,7 +532,7 @@
 passages are candidates; check relevance before using them as evidence.</t>
   </si>
   <si>
-    <t>01a0d585-0187-7fd1-8aaf-ce8e103bf520</t>
+    <t>01a1143f-aaa2-76c3-807c-e7d56fd0d3c8</t>
   </si>
 </sst>
 </file>
@@ -859,7 +939,7 @@
   <sheetPr>
     <tabColor rgb="FF173B70"/>
   </sheetPr>
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="10.7109375" customWidth="1"/>
@@ -916,23 +996,23 @@
     </row>
     <row r="2" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
       <c r="C2" s="4" t="s">
-        <v>91</v>
+        <v>122</v>
       </c>
       <c r="E2" s="2">
-        <f>IF(COUNT('Turns'!E17,'Turns'!E32)=2,SUM('Turns'!E17,'Turns'!E32),"Unknown")</f>
-        <v>0.001091537405</v>
+        <f>IF(COUNT('Turns'!E16,'Turns'!E31)=2,SUM('Turns'!E16,'Turns'!E31),"Unknown")</f>
+        <v>0.0004432306068</v>
       </c>
       <c r="F2" s="2">
-        <f>IF(COUNT('Turns'!F17,'Turns'!F32)=2,SUM('Turns'!F17,'Turns'!F32),"Unknown")</f>
-        <v>0.00124075</v>
+        <f>IF(COUNT('Turns'!F16,'Turns'!F31)=2,SUM('Turns'!F16,'Turns'!F31),"Unknown")</f>
+        <v>0.00050382</v>
       </c>
       <c r="G2" s="5">
         <f>IF(ISNUMBER(E2),ROUND(E2*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>109.0</v>
+        <v>44.0</v>
       </c>
       <c r="H2" s="5">
         <f>IF(ISNUMBER(F2),ROUND(F2*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>124.0</v>
+        <v>50.0</v>
       </c>
     </row>
     <row r="3" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
@@ -940,578 +1020,558 @@
         <v>1</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
       <c r="E3" s="2">
-        <f>IF(COUNT('Turns'!E17,'Turns'!E32)=2,SUM('Turns'!E17,'Turns'!E32),"Unknown")</f>
-        <v>0.001091537405</v>
+        <f>IF(COUNT('Turns'!E16,'Turns'!E31)=2,SUM('Turns'!E16,'Turns'!E31),"Unknown")</f>
+        <v>0.0004432306068</v>
       </c>
       <c r="F3" s="2">
-        <f>IF(COUNT('Turns'!F17,'Turns'!F32)=2,SUM('Turns'!F17,'Turns'!F32),"Unknown")</f>
-        <v>0.00124075</v>
+        <f>IF(COUNT('Turns'!F16,'Turns'!F31)=2,SUM('Turns'!F16,'Turns'!F31),"Unknown")</f>
+        <v>0.00050382</v>
       </c>
       <c r="G3" s="5">
         <f>IF(ISNUMBER(E3),ROUND(E3*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>109.0</v>
+        <v>44.0</v>
       </c>
       <c r="H3" s="5">
         <f>IF(ISNUMBER(F3),ROUND(F3*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>124.0</v>
+        <v>50.0</v>
       </c>
     </row>
     <row r="4" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="B4" s="4">
         <v>1</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="D4" s="4">
-        <v>2123</v>
+        <v>244</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>96</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="24" customHeight="1">
       <c r="A5" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>97</v>
+        <v>128</v>
       </c>
       <c r="D5" s="5">
-        <v>3</v>
+        <v>244</v>
       </c>
       <c r="E5" s="2">
         <f>IF(AND(ISNUMBER(F5),ISNUMBER('Reference data'!$B$3)),F5*'Reference data'!$B$3,"Unknown")</f>
-        <v>5.27844e-07</v>
+        <v>4.2931312e-05</v>
       </c>
       <c r="F5" s="2">
-        <f>IF(D5=0,0,IF(ISNUMBER('Reference data'!B17),D5*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>6e-07</v>
+        <f>IF(D5=0,0,IF(ISNUMBER('Reference data'!B22),D5*'Reference data'!B22/1000000,"Unknown"))</f>
+        <v>4.88e-05</v>
       </c>
       <c r="G5" s="5">
         <f>IF(ISNUMBER(E5),ROUND(E5*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="H5" s="5">
         <f>IF(ISNUMBER(F5),ROUND(F5*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>0.0</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="24" customHeight="1">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>98</v>
+        <v>129</v>
+      </c>
+      <c r="D6" s="1">
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="73" customHeight="1">
       <c r="A7" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>130</v>
+      </c>
+      <c r="D7" s="1">
+        <v>87</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>100</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="24" customHeight="1">
       <c r="A8" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>101</v>
+        <v>132</v>
+      </c>
+      <c r="D8" s="1">
+        <v>33</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>102</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="24" customHeight="1">
       <c r="A9" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>103</v>
-      </c>
-      <c r="D9" s="5">
-        <v>2120</v>
-      </c>
-      <c r="E9" s="2">
-        <f>IF(AND(ISNUMBER(F9),ISNUMBER('Reference data'!$B$3)),F9*'Reference data'!$B$3,"Unknown")</f>
-        <v>0.0004662622</v>
-      </c>
-      <c r="F9" s="2">
-        <f>IF(D9=0,0,IF(ISNUMBER('Reference data'!D17),D9*'Reference data'!D17/1000000,"Unknown"))</f>
-        <v>0.00053</v>
-      </c>
-      <c r="G9" s="5">
-        <f>IF(ISNUMBER(E9),ROUND(E9*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>47.0</v>
-      </c>
-      <c r="H9" s="5">
-        <f>IF(ISNUMBER(F9),ROUND(F9*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>53.0</v>
+        <v>134</v>
+      </c>
+      <c r="D9" s="1">
+        <v>244</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="24" customHeight="1">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>104</v>
+        <v>135</v>
+      </c>
+      <c r="D10" s="1">
+        <v>244</v>
+      </c>
+      <c r="L10" s="1">
+        <v>244</v>
       </c>
     </row>
     <row r="11" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="B11" s="4">
         <v>1</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
       <c r="D11" s="4">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="24" customHeight="1">
       <c r="A12" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>106</v>
+        <v>137</v>
       </c>
       <c r="D12" s="5">
-        <v>11</v>
+        <v>67</v>
       </c>
       <c r="E12" s="2">
         <f>IF(AND(ISNUMBER(F12),ISNUMBER('Reference data'!$B$3)),F12*'Reference data'!$B$3,"Unknown")</f>
-        <v>1.1612568e-05</v>
+        <v>7.0731096e-05</v>
       </c>
       <c r="F12" s="2">
-        <f>IF(D12=0,0,IF(ISNUMBER('Reference data'!F17),D12*'Reference data'!F17/1000000,"Unknown"))</f>
-        <v>1.32e-05</v>
+        <f>IF(D12=0,0,IF(ISNUMBER('Reference data'!E22),D12*'Reference data'!E22/1000000,"Unknown"))</f>
+        <v>8.04e-05</v>
       </c>
       <c r="G12" s="5">
         <f>IF(ISNUMBER(E12),ROUND(E12*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>1.0</v>
+        <v>7.0</v>
       </c>
       <c r="H12" s="5">
         <f>IF(ISNUMBER(F12),ROUND(F12*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="24" customHeight="1">
+        <v>8.0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="34" customHeight="1">
       <c r="A13" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>107</v>
-      </c>
-      <c r="D13" s="5">
-        <v>43</v>
-      </c>
-      <c r="E13" s="2">
-        <f>IF(AND(ISNUMBER(F13),ISNUMBER('Reference data'!$B$3)),F13*'Reference data'!$B$3,"Unknown")</f>
-        <v>4.5394584e-05</v>
-      </c>
-      <c r="F13" s="2">
-        <f>IF(D13=0,0,IF(ISNUMBER('Reference data'!E17),D13*'Reference data'!E17/1000000,"Unknown"))</f>
-        <v>5.16e-05</v>
-      </c>
-      <c r="G13" s="5">
-        <f>IF(ISNUMBER(E13),ROUND(E13*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>5.0</v>
-      </c>
-      <c r="H13" s="5">
-        <f>IF(ISNUMBER(F13),ROUND(F13*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="307" customHeight="1">
+        <v>138</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="24" customHeight="1">
       <c r="A14" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>108</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>109</v>
+        <v>134</v>
+      </c>
+      <c r="D14" s="1">
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="24" customHeight="1">
       <c r="A15" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="24" customHeight="1">
-      <c r="A16" t="s">
-        <v>93</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-      <c r="C16" t="s">
-        <v>104</v>
+        <v>135</v>
+      </c>
+      <c r="D15" s="1">
+        <v>67</v>
+      </c>
+      <c r="L15" s="1">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
+      <c r="A16" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B16" s="4">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="E16" s="2">
+        <f>IF(COUNT('Turns'!E5,'Turns'!E12)=2,SUM('Turns'!E5,'Turns'!E12),"Unknown")</f>
+        <v>0.000113662408</v>
+      </c>
+      <c r="F16" s="2">
+        <f>IF(COUNT('Turns'!F5,'Turns'!F12)=2,SUM('Turns'!F5,'Turns'!F12),"Unknown")</f>
+        <v>0.0001292</v>
+      </c>
+      <c r="G16" s="5">
+        <f>IF(ISNUMBER(E16),ROUND(E16*'Reference data'!$B$2,0),"Unknown")</f>
+        <v>11.0</v>
+      </c>
+      <c r="H16" s="5">
+        <f>IF(ISNUMBER(F16),ROUND(F16*'Reference data'!$B$2,0),"Unknown")</f>
+        <v>13.0</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="17" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
-      <c r="A17" s="4" t="s">
-        <v>93</v>
-      </c>
       <c r="B17" s="4">
         <v>1</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="E17" s="2">
-        <f>IF(COUNT('Turns'!E5,'Turns'!E9,'Turns'!E12,'Turns'!E13)=4,SUM('Turns'!E5,'Turns'!E9,'Turns'!E12,'Turns'!E13),"Unknown")</f>
-        <v>0.000523797196</v>
-      </c>
-      <c r="F17" s="2">
-        <f>IF(COUNT('Turns'!F5,'Turns'!F9,'Turns'!F12,'Turns'!F13)=4,SUM('Turns'!F5,'Turns'!F9,'Turns'!F12,'Turns'!F13),"Unknown")</f>
-        <v>0.0005954</v>
-      </c>
-      <c r="G17" s="5">
-        <f>IF(ISNUMBER(E17),ROUND(E17*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>52.0</v>
-      </c>
-      <c r="H17" s="5">
-        <f>IF(ISNUMBER(F17),ROUND(F17*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>60.0</v>
+        <v>142</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
-      <c r="B18" s="4">
-        <v>1</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="M18" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="34" customHeight="1">
+        <v>141</v>
+      </c>
+      <c r="M17" s="4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="24" customHeight="1">
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
+        <v>144</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="409" customHeight="1">
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>114</v>
+        <v>146</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" ht="409" customHeight="1">
-      <c r="B20">
-        <v>1</v>
-      </c>
-      <c r="C20" t="s">
-        <v>116</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
-      <c r="A21" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B21" s="4">
-        <v>1</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D21" s="4">
-        <v>3630</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="M21" s="4" t="s">
-        <v>119</v>
+        <v>147</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
+      <c r="A20" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B20" s="4">
+        <v>1</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D20" s="4">
+        <v>1829</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="24" customHeight="1">
+      <c r="A21" t="s">
+        <v>148</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>150</v>
+      </c>
+      <c r="D21" s="5">
+        <v>311</v>
+      </c>
+      <c r="E21" s="2">
+        <f>IF(AND(ISNUMBER(F21),ISNUMBER('Reference data'!$B$3)),F21*'Reference data'!$B$3,"Unknown")</f>
+        <v>5.4719828e-06</v>
+      </c>
+      <c r="F21" s="2">
+        <f>IF(D21=0,0,IF(ISNUMBER('Reference data'!C22),D21*'Reference data'!C22/1000000,"Unknown"))</f>
+        <v>6.22e-06</v>
+      </c>
+      <c r="G21" s="5">
+        <f>IF(ISNUMBER(E21),ROUND(E21*'Reference data'!$B$2,0),"Unknown")</f>
+        <v>1.0</v>
+      </c>
+      <c r="H21" s="5">
+        <f>IF(ISNUMBER(F21),ROUND(F21*'Reference data'!$B$2,0),"Unknown")</f>
+        <v>1.0</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="24" customHeight="1">
       <c r="A22" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="D22" s="5">
-        <v>2120</v>
+        <v>1518</v>
       </c>
       <c r="E22" s="2">
         <f>IF(AND(ISNUMBER(F22),ISNUMBER('Reference data'!$B$3)),F22*'Reference data'!$B$3,"Unknown")</f>
-        <v>3.7300976e-05</v>
+        <v>0.000267089064</v>
       </c>
       <c r="F22" s="2">
-        <f>IF(D22=0,0,IF(ISNUMBER('Reference data'!C17),D22*'Reference data'!C17/1000000,"Unknown"))</f>
-        <v>4.24e-05</v>
+        <f>IF(D22=0,0,IF(ISNUMBER('Reference data'!B22),D22*'Reference data'!B22/1000000,"Unknown"))</f>
+        <v>0.0003036</v>
       </c>
       <c r="G22" s="5">
         <f>IF(ISNUMBER(E22),ROUND(E22*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>4.0</v>
+        <v>27.0</v>
       </c>
       <c r="H22" s="5">
         <f>IF(ISNUMBER(F22),ROUND(F22*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" ht="24" customHeight="1">
+        <v>30.0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="409" customHeight="1">
       <c r="A23" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>97</v>
-      </c>
-      <c r="D23" s="5">
-        <v>3</v>
-      </c>
-      <c r="E23" s="2">
-        <f>IF(AND(ISNUMBER(F23),ISNUMBER('Reference data'!$B$3)),F23*'Reference data'!$B$3,"Unknown")</f>
-        <v>5.27844e-07</v>
-      </c>
-      <c r="F23" s="2">
-        <f>IF(D23=0,0,IF(ISNUMBER('Reference data'!B17),D23*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>6e-07</v>
-      </c>
-      <c r="G23" s="5">
-        <f>IF(ISNUMBER(E23),ROUND(E23*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>0.0</v>
-      </c>
-      <c r="H23" s="5">
-        <f>IF(ISNUMBER(F23),ROUND(F23*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" ht="409" customHeight="1">
+        <v>151</v>
+      </c>
+      <c r="D23" s="1">
+        <v>1518</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="24" customHeight="1">
       <c r="A24" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="B24">
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>121</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>117</v>
+        <v>134</v>
+      </c>
+      <c r="D24" s="1">
+        <v>1518</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="24" customHeight="1">
       <c r="A25" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="B25">
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>103</v>
-      </c>
-      <c r="D25" s="5">
-        <v>1507</v>
-      </c>
-      <c r="E25" s="2">
-        <f>IF(AND(ISNUMBER(F25),ISNUMBER('Reference data'!$B$3)),F25*'Reference data'!$B$3,"Unknown")</f>
-        <v>0.000331442045</v>
-      </c>
-      <c r="F25" s="2">
-        <f>IF(D25=0,0,IF(ISNUMBER('Reference data'!D17),D25*'Reference data'!D17/1000000,"Unknown"))</f>
-        <v>0.00037675</v>
-      </c>
-      <c r="G25" s="5">
-        <f>IF(ISNUMBER(E25),ROUND(E25*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>33.0</v>
-      </c>
-      <c r="H25" s="5">
-        <f>IF(ISNUMBER(F25),ROUND(F25*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>38.0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" ht="24" customHeight="1">
-      <c r="A26" t="s">
-        <v>118</v>
-      </c>
-      <c r="B26">
-        <v>1</v>
-      </c>
-      <c r="C26" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
-      <c r="A27" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B27" s="4">
-        <v>1</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="D27" s="4">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" ht="24" customHeight="1">
+        <v>135</v>
+      </c>
+      <c r="D25" s="1">
+        <v>1518</v>
+      </c>
+      <c r="L25" s="1">
+        <v>1829</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
+      <c r="A26" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B26" s="4">
+        <v>1</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D26" s="4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="24" customHeight="1">
+      <c r="A27" t="s">
+        <v>148</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>137</v>
+      </c>
+      <c r="D27" s="5">
+        <v>54</v>
+      </c>
+      <c r="E27" s="2">
+        <f>IF(AND(ISNUMBER(F27),ISNUMBER('Reference data'!$B$3)),F27*'Reference data'!$B$3,"Unknown")</f>
+        <v>5.7007152e-05</v>
+      </c>
+      <c r="F27" s="2">
+        <f>IF(D27=0,0,IF(ISNUMBER('Reference data'!E22),D27*'Reference data'!E22/1000000,"Unknown"))</f>
+        <v>6.48e-05</v>
+      </c>
+      <c r="G27" s="5">
+        <f>IF(ISNUMBER(E27),ROUND(E27*'Reference data'!$B$2,0),"Unknown")</f>
+        <v>6.0</v>
+      </c>
+      <c r="H27" s="5">
+        <f>IF(ISNUMBER(F27),ROUND(F27*'Reference data'!$B$2,0),"Unknown")</f>
+        <v>6.0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" ht="47" customHeight="1">
       <c r="A28" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="B28">
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>107</v>
-      </c>
-      <c r="D28" s="5">
-        <v>188</v>
-      </c>
-      <c r="E28" s="2">
-        <f>IF(AND(ISNUMBER(F28),ISNUMBER('Reference data'!$B$3)),F28*'Reference data'!$B$3,"Unknown")</f>
-        <v>0.000198469344</v>
-      </c>
-      <c r="F28" s="2">
-        <f>IF(D28=0,0,IF(ISNUMBER('Reference data'!E17),D28*'Reference data'!E17/1000000,"Unknown"))</f>
-        <v>0.0002256</v>
-      </c>
-      <c r="G28" s="5">
-        <f>IF(ISNUMBER(E28),ROUND(E28*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>20.0</v>
-      </c>
-      <c r="H28" s="5">
-        <f>IF(ISNUMBER(F28),ROUND(F28*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>23.0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" ht="164" customHeight="1">
+        <v>138</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="24" customHeight="1">
       <c r="A29" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="B29">
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>108</v>
-      </c>
-      <c r="I29" s="6" t="s">
-        <v>122</v>
+        <v>134</v>
+      </c>
+      <c r="D29" s="1">
+        <v>54</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="24" customHeight="1">
       <c r="A30" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" ht="24" customHeight="1">
-      <c r="A31" t="s">
-        <v>118</v>
-      </c>
-      <c r="B31">
-        <v>1</v>
-      </c>
-      <c r="C31" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
-      <c r="A32" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B32" s="4">
-        <v>1</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="E32" s="2">
-        <f>IF(COUNT('Turns'!E22,'Turns'!E23,'Turns'!E25,'Turns'!E28)=4,SUM('Turns'!E22,'Turns'!E23,'Turns'!E25,'Turns'!E28),"Unknown")</f>
-        <v>0.000567740209</v>
-      </c>
-      <c r="F32" s="2">
-        <f>IF(COUNT('Turns'!F22,'Turns'!F23,'Turns'!F25,'Turns'!F28)=4,SUM('Turns'!F22,'Turns'!F23,'Turns'!F25,'Turns'!F28),"Unknown")</f>
-        <v>0.00064535</v>
-      </c>
-      <c r="G32" s="5">
-        <f>IF(ISNUMBER(E32),ROUND(E32*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>57.0</v>
-      </c>
-      <c r="H32" s="5">
-        <f>IF(ISNUMBER(F32),ROUND(F32*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>65.0</v>
-      </c>
-      <c r="K32" s="4" t="s">
-        <v>111</v>
+        <v>135</v>
+      </c>
+      <c r="D30" s="1">
+        <v>54</v>
+      </c>
+      <c r="L30" s="1">
+        <v>1883</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
+      <c r="A31" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B31" s="4">
+        <v>1</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="E31" s="2">
+        <f>IF(COUNT('Turns'!E21,'Turns'!E22,'Turns'!E27)=3,SUM('Turns'!E21,'Turns'!E22,'Turns'!E27),"Unknown")</f>
+        <v>0.0003295681988</v>
+      </c>
+      <c r="F31" s="2">
+        <f>IF(COUNT('Turns'!F21,'Turns'!F22,'Turns'!F27)=3,SUM('Turns'!F21,'Turns'!F22,'Turns'!F27),"Unknown")</f>
+        <v>0.00037462</v>
+      </c>
+      <c r="G31" s="5">
+        <f>IF(ISNUMBER(E31),ROUND(E31*'Reference data'!$B$2,0),"Unknown")</f>
+        <v>33.0</v>
+      </c>
+      <c r="H31" s="5">
+        <f>IF(ISNUMBER(F31),ROUND(F31*'Reference data'!$B$2,0),"Unknown")</f>
+        <v>37.0</v>
+      </c>
+      <c r="K31" s="4" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:AE32">
+  <conditionalFormatting sqref="A2:AE31">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$K2="error"</formula>
     </cfRule>
@@ -1525,7 +1585,7 @@
   <sheetPr>
     <tabColor rgb="FF173B70"/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="48.7109375" customWidth="1"/>
@@ -1632,177 +1692,241 @@
     </row>
     <row r="2" spans="1:31" ht="54" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>123</v>
+        <v>153</v>
       </c>
       <c r="B2" s="1">
         <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>111</v>
+        <v>141</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>125</v>
+        <v>155</v>
       </c>
       <c r="H2" t="s">
         <v>49</v>
       </c>
       <c r="J2" s="2">
-        <f>IF(COUNT('Turns'!D5,'Turns'!D23)=2,SUM('Turns'!D5,'Turns'!D23),"Unknown")</f>
-        <v>6.0</v>
+        <f>IF(COUNT('Turns'!D5,'Turns'!D22)=2,SUM('Turns'!D5,'Turns'!D22),"Unknown")</f>
+        <v>1762.0</v>
       </c>
       <c r="K2" s="2">
-        <f>IF(COUNT('Turns'!E5,'Turns'!E23)=2,SUM('Turns'!E5,'Turns'!E23),"Unknown")</f>
-        <v>1.055688e-06</v>
+        <f>IF(COUNT('Turns'!E5,'Turns'!E22)=2,SUM('Turns'!E5,'Turns'!E22),"Unknown")</f>
+        <v>0.000310020376</v>
       </c>
       <c r="L2" s="2">
-        <f>IF(COUNT('Turns'!F5,'Turns'!F23)=2,SUM('Turns'!F5,'Turns'!F23),"Unknown")</f>
-        <v>1.2e-06</v>
+        <f>IF(COUNT('Turns'!F5,'Turns'!F22)=2,SUM('Turns'!F5,'Turns'!F22),"Unknown")</f>
+        <v>0.0003524</v>
       </c>
       <c r="M2" s="2">
-        <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
-        <v>2120.0</v>
+        <f>IF(COUNT('Turns'!D21)=1,SUM('Turns'!D21),"Unknown")</f>
+        <v>311.0</v>
       </c>
       <c r="N2" s="2">
-        <f>IF(COUNT('Turns'!E22)=1,SUM('Turns'!E22),"Unknown")</f>
-        <v>3.7300976e-05</v>
+        <f>IF(COUNT('Turns'!E21)=1,SUM('Turns'!E21),"Unknown")</f>
+        <v>5.4719828e-06</v>
       </c>
       <c r="O2" s="2">
-        <f>IF(COUNT('Turns'!F22)=1,SUM('Turns'!F22),"Unknown")</f>
-        <v>4.24e-05</v>
+        <f>IF(COUNT('Turns'!F21)=1,SUM('Turns'!F21),"Unknown")</f>
+        <v>6.22e-06</v>
       </c>
       <c r="P2" s="2">
-        <f>IF(COUNT('Turns'!D9,'Turns'!D25)=2,SUM('Turns'!D9,'Turns'!D25),"Unknown")</f>
-        <v>3627.0</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="2">
-        <f>IF(COUNT('Turns'!E9,'Turns'!E25)=2,SUM('Turns'!E9,'Turns'!E25),"Unknown")</f>
-        <v>0.000797704245</v>
+        <v>0</v>
       </c>
       <c r="R2" s="2">
-        <f>IF(COUNT('Turns'!F9,'Turns'!F25)=2,SUM('Turns'!F9,'Turns'!F25),"Unknown")</f>
-        <v>0.00090675</v>
+        <v>0</v>
       </c>
       <c r="S2" s="2">
-        <f>IF(COUNT('Turns'!D13,'Turns'!D28)=2,SUM('Turns'!D13,'Turns'!D28),"Unknown")</f>
-        <v>231.0</v>
+        <f>IF(COUNT('Turns'!D12,'Turns'!D27)=2,SUM('Turns'!D12,'Turns'!D27),"Unknown")</f>
+        <v>121.0</v>
       </c>
       <c r="T2" s="2">
-        <f>IF(COUNT('Turns'!E13,'Turns'!E28)=2,SUM('Turns'!E13,'Turns'!E28),"Unknown")</f>
-        <v>0.000243863928</v>
+        <f>IF(COUNT('Turns'!E12,'Turns'!E27)=2,SUM('Turns'!E12,'Turns'!E27),"Unknown")</f>
+        <v>0.000127738248</v>
       </c>
       <c r="U2" s="2">
-        <f>IF(COUNT('Turns'!F13,'Turns'!F28)=2,SUM('Turns'!F13,'Turns'!F28),"Unknown")</f>
-        <v>0.0002772</v>
+        <f>IF(COUNT('Turns'!F12,'Turns'!F27)=2,SUM('Turns'!F12,'Turns'!F27),"Unknown")</f>
+        <v>0.0001452</v>
       </c>
       <c r="V2" s="2">
-        <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>11.0</v>
+        <v>0</v>
       </c>
       <c r="W2" s="2">
-        <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.1612568e-05</v>
+        <v>0</v>
       </c>
       <c r="X2" s="2">
-        <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.32e-05</v>
+        <v>0</v>
       </c>
       <c r="Y2" s="2">
-        <f>IF(COUNT('Turns'!E17,'Turns'!E32)=2,SUM('Turns'!E17,'Turns'!E32),"Unknown")</f>
-        <v>0.001091537405</v>
+        <f>IF(COUNT('Turns'!E16,'Turns'!E31)=2,SUM('Turns'!E16,'Turns'!E31),"Unknown")</f>
+        <v>0.0004432306068</v>
       </c>
       <c r="Z2" s="2">
-        <f>IF(COUNT('Turns'!F17,'Turns'!F32)=2,SUM('Turns'!F17,'Turns'!F32),"Unknown")</f>
-        <v>0.00124075</v>
+        <f>IF(COUNT('Turns'!F16,'Turns'!F31)=2,SUM('Turns'!F16,'Turns'!F31),"Unknown")</f>
+        <v>0.00050382</v>
       </c>
       <c r="AA2" s="5">
         <f>IF(ISNUMBER(Y2),ROUND(Y2*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>109.0</v>
+        <v>44.0</v>
       </c>
       <c r="AB2" s="5">
         <f>IF(ISNUMBER(Z2),ROUND(Z2*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>124.0</v>
+        <v>50.0</v>
       </c>
       <c r="AD2" s="1">
-        <v>5773.972</v>
+        <v>451.639</v>
       </c>
       <c r="AE2" s="1" t="s">
-        <v>126</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:31" ht="54" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>111</v>
+        <v>141</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>128</v>
+        <v>158</v>
       </c>
       <c r="H3" t="s">
-        <v>129</v>
+        <v>159</v>
       </c>
       <c r="I3" t="s">
         <v>49</v>
       </c>
+      <c r="J3" s="2">
+        <f>IF(COUNT('Turns'!D5)=1,SUM('Turns'!D5),"Unknown")</f>
+        <v>244.0</v>
+      </c>
+      <c r="K3" s="2">
+        <f>IF(COUNT('Turns'!E5)=1,SUM('Turns'!E5),"Unknown")</f>
+        <v>4.2931312e-05</v>
+      </c>
+      <c r="L3" s="2">
+        <f>IF(COUNT('Turns'!F5)=1,SUM('Turns'!F5),"Unknown")</f>
+        <v>4.88e-05</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0</v>
+      </c>
+      <c r="N3" s="2">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2">
+        <v>0</v>
+      </c>
+      <c r="P3" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>0</v>
+      </c>
+      <c r="R3" s="2">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2">
+        <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
+        <v>67.0</v>
+      </c>
+      <c r="T3" s="2">
+        <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
+        <v>7.0731096e-05</v>
+      </c>
+      <c r="U3" s="2">
+        <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
+        <v>8.04e-05</v>
+      </c>
+      <c r="V3" s="2">
+        <v>0</v>
+      </c>
+      <c r="W3" s="2">
+        <v>0</v>
+      </c>
+      <c r="X3" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="2">
+        <f>IF(COUNT('Turns'!E16)=1,SUM('Turns'!E16),"Unknown")</f>
+        <v>0.000113662408</v>
+      </c>
+      <c r="Z3" s="2">
+        <f>IF(COUNT('Turns'!F16)=1,SUM('Turns'!F16),"Unknown")</f>
+        <v>0.0001292</v>
+      </c>
+      <c r="AA3" s="5">
+        <f>IF(ISNUMBER(Y3),ROUND(Y3*'Reference data'!$B$2,0),"Unknown")</f>
+        <v>11.0</v>
+      </c>
+      <c r="AB3" s="5">
+        <f>IF(ISNUMBER(Z3),ROUND(Z3*'Reference data'!$B$2,0),"Unknown")</f>
+        <v>13.0</v>
+      </c>
       <c r="AD3" s="1">
-        <v>0.989</v>
+        <v>130.569</v>
       </c>
       <c r="AE3" s="1" t="s">
-        <v>130</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:31" ht="54" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>131</v>
+        <v>160</v>
       </c>
       <c r="B4" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>124</v>
+        <v>161</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>47</v>
+        <v>126</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>111</v>
+        <v>141</v>
+      </c>
+      <c r="F4" s="1">
+        <v>244</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>132</v>
+        <v>162</v>
       </c>
       <c r="H4" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="I4" t="s">
-        <v>49</v>
+        <v>159</v>
       </c>
       <c r="J4" s="2">
         <f>IF(COUNT('Turns'!D5)=1,SUM('Turns'!D5),"Unknown")</f>
-        <v>3.0</v>
+        <v>244.0</v>
       </c>
       <c r="K4" s="2">
         <f>IF(COUNT('Turns'!E5)=1,SUM('Turns'!E5),"Unknown")</f>
-        <v>5.27844e-07</v>
+        <v>4.2931312e-05</v>
       </c>
       <c r="L4" s="2">
         <f>IF(COUNT('Turns'!F5)=1,SUM('Turns'!F5),"Unknown")</f>
-        <v>6e-07</v>
+        <v>4.88e-05</v>
       </c>
       <c r="M4" s="2">
         <v>0</v>
@@ -1814,311 +1938,299 @@
         <v>0</v>
       </c>
       <c r="P4" s="2">
-        <f>IF(COUNT('Turns'!D9)=1,SUM('Turns'!D9),"Unknown")</f>
-        <v>2120.0</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="2">
-        <f>IF(COUNT('Turns'!E9)=1,SUM('Turns'!E9),"Unknown")</f>
-        <v>0.0004662622</v>
+        <v>0</v>
       </c>
       <c r="R4" s="2">
-        <f>IF(COUNT('Turns'!F9)=1,SUM('Turns'!F9),"Unknown")</f>
-        <v>0.00053</v>
+        <v>0</v>
       </c>
       <c r="S4" s="2">
-        <f>IF(COUNT('Turns'!D13)=1,SUM('Turns'!D13),"Unknown")</f>
-        <v>43.0</v>
+        <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
+        <v>67.0</v>
       </c>
       <c r="T4" s="2">
-        <f>IF(COUNT('Turns'!E13)=1,SUM('Turns'!E13),"Unknown")</f>
-        <v>4.5394584e-05</v>
+        <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
+        <v>7.0731096e-05</v>
       </c>
       <c r="U4" s="2">
-        <f>IF(COUNT('Turns'!F13)=1,SUM('Turns'!F13),"Unknown")</f>
-        <v>5.16e-05</v>
+        <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
+        <v>8.04e-05</v>
       </c>
       <c r="V4" s="2">
-        <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>11.0</v>
+        <v>0</v>
       </c>
       <c r="W4" s="2">
-        <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.1612568e-05</v>
+        <v>0</v>
       </c>
       <c r="X4" s="2">
-        <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.32e-05</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="2">
-        <f>IF(COUNT('Turns'!E17)=1,SUM('Turns'!E17),"Unknown")</f>
-        <v>0.000523797196</v>
+        <f>IF(COUNT('Turns'!E16)=1,SUM('Turns'!E16),"Unknown")</f>
+        <v>0.000113662408</v>
       </c>
       <c r="Z4" s="2">
-        <f>IF(COUNT('Turns'!F17)=1,SUM('Turns'!F17),"Unknown")</f>
-        <v>0.0005954</v>
+        <f>IF(COUNT('Turns'!F16)=1,SUM('Turns'!F16),"Unknown")</f>
+        <v>0.0001292</v>
       </c>
       <c r="AA4" s="5">
         <f>IF(ISNUMBER(Y4),ROUND(Y4*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>52.0</v>
+        <v>11.0</v>
       </c>
       <c r="AB4" s="5">
         <f>IF(ISNUMBER(Z4),ROUND(Z4*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>60.0</v>
+        <v>13.0</v>
+      </c>
+      <c r="AC4" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="AD4" s="1">
-        <v>1651.68</v>
+        <v>129.138</v>
       </c>
       <c r="AE4" s="1" t="s">
-        <v>126</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:31" ht="54" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>134</v>
+        <v>164</v>
       </c>
       <c r="B5" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>95</v>
+        <v>47</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F5" s="1">
-        <v>2123</v>
+        <v>141</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>136</v>
+        <v>165</v>
       </c>
       <c r="H5" t="s">
-        <v>96</v>
+        <v>166</v>
       </c>
       <c r="I5" t="s">
-        <v>133</v>
-      </c>
-      <c r="J5" s="2">
-        <f>IF(COUNT('Turns'!D5)=1,SUM('Turns'!D5),"Unknown")</f>
-        <v>3.0</v>
-      </c>
-      <c r="K5" s="2">
-        <f>IF(COUNT('Turns'!E5)=1,SUM('Turns'!E5),"Unknown")</f>
-        <v>5.27844e-07</v>
-      </c>
-      <c r="L5" s="2">
-        <f>IF(COUNT('Turns'!F5)=1,SUM('Turns'!F5),"Unknown")</f>
-        <v>6e-07</v>
-      </c>
-      <c r="M5" s="2">
-        <v>0</v>
-      </c>
-      <c r="N5" s="2">
-        <v>0</v>
-      </c>
-      <c r="O5" s="2">
-        <v>0</v>
-      </c>
-      <c r="P5" s="2">
-        <f>IF(COUNT('Turns'!D9)=1,SUM('Turns'!D9),"Unknown")</f>
-        <v>2120.0</v>
-      </c>
-      <c r="Q5" s="2">
-        <f>IF(COUNT('Turns'!E9)=1,SUM('Turns'!E9),"Unknown")</f>
-        <v>0.0004662622</v>
-      </c>
-      <c r="R5" s="2">
-        <f>IF(COUNT('Turns'!F9)=1,SUM('Turns'!F9),"Unknown")</f>
-        <v>0.00053</v>
-      </c>
-      <c r="S5" s="2">
-        <f>IF(COUNT('Turns'!D13)=1,SUM('Turns'!D13),"Unknown")</f>
-        <v>43.0</v>
-      </c>
-      <c r="T5" s="2">
-        <f>IF(COUNT('Turns'!E13)=1,SUM('Turns'!E13),"Unknown")</f>
-        <v>4.5394584e-05</v>
-      </c>
-      <c r="U5" s="2">
-        <f>IF(COUNT('Turns'!F13)=1,SUM('Turns'!F13),"Unknown")</f>
-        <v>5.16e-05</v>
-      </c>
-      <c r="V5" s="2">
-        <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>11.0</v>
-      </c>
-      <c r="W5" s="2">
-        <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.1612568e-05</v>
-      </c>
-      <c r="X5" s="2">
-        <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.32e-05</v>
-      </c>
-      <c r="Y5" s="2">
-        <f>IF(COUNT('Turns'!E17)=1,SUM('Turns'!E17),"Unknown")</f>
-        <v>0.000523797196</v>
-      </c>
-      <c r="Z5" s="2">
-        <f>IF(COUNT('Turns'!F17)=1,SUM('Turns'!F17),"Unknown")</f>
-        <v>0.0005954</v>
-      </c>
-      <c r="AA5" s="5">
-        <f>IF(ISNUMBER(Y5),ROUND(Y5*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>52.0</v>
-      </c>
-      <c r="AB5" s="5">
-        <f>IF(ISNUMBER(Z5),ROUND(Z5*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>60.0</v>
-      </c>
-      <c r="AC5" s="1" t="s">
-        <v>93</v>
+        <v>49</v>
       </c>
       <c r="AD5" s="1">
-        <v>1634.994</v>
+        <v>314.711</v>
       </c>
       <c r="AE5" s="1" t="s">
-        <v>137</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:31" ht="54" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>138</v>
+        <v>168</v>
       </c>
       <c r="B6" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>124</v>
+        <v>169</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>111</v>
+        <v>141</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>139</v>
+        <v>170</v>
       </c>
       <c r="H6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="I6" t="s">
-        <v>49</v>
+        <v>166</v>
       </c>
       <c r="AD6" s="1">
-        <v>1236.595</v>
+        <v>313.632</v>
       </c>
       <c r="AE6" s="1" t="s">
-        <v>130</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7" spans="1:31" ht="54" customHeight="1">
       <c r="A7" s="6" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="B7" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>111</v>
+        <v>141</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="H7" t="s">
-        <v>113</v>
+        <v>171</v>
       </c>
       <c r="I7" t="s">
-        <v>140</v>
+        <v>49</v>
+      </c>
+      <c r="J7" s="2">
+        <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
+        <v>1518.0</v>
+      </c>
+      <c r="K7" s="2">
+        <f>IF(COUNT('Turns'!E22)=1,SUM('Turns'!E22),"Unknown")</f>
+        <v>0.000267089064</v>
+      </c>
+      <c r="L7" s="2">
+        <f>IF(COUNT('Turns'!F22)=1,SUM('Turns'!F22),"Unknown")</f>
+        <v>0.0003036</v>
+      </c>
+      <c r="M7" s="2">
+        <f>IF(COUNT('Turns'!D21)=1,SUM('Turns'!D21),"Unknown")</f>
+        <v>311.0</v>
+      </c>
+      <c r="N7" s="2">
+        <f>IF(COUNT('Turns'!E21)=1,SUM('Turns'!E21),"Unknown")</f>
+        <v>5.4719828e-06</v>
+      </c>
+      <c r="O7" s="2">
+        <f>IF(COUNT('Turns'!F21)=1,SUM('Turns'!F21),"Unknown")</f>
+        <v>6.22e-06</v>
+      </c>
+      <c r="P7" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>0</v>
+      </c>
+      <c r="R7" s="2">
+        <v>0</v>
+      </c>
+      <c r="S7" s="2">
+        <f>IF(COUNT('Turns'!D27)=1,SUM('Turns'!D27),"Unknown")</f>
+        <v>54.0</v>
+      </c>
+      <c r="T7" s="2">
+        <f>IF(COUNT('Turns'!E27)=1,SUM('Turns'!E27),"Unknown")</f>
+        <v>5.7007152e-05</v>
+      </c>
+      <c r="U7" s="2">
+        <f>IF(COUNT('Turns'!F27)=1,SUM('Turns'!F27),"Unknown")</f>
+        <v>6.48e-05</v>
+      </c>
+      <c r="V7" s="2">
+        <v>0</v>
+      </c>
+      <c r="W7" s="2">
+        <v>0</v>
+      </c>
+      <c r="X7" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="2">
+        <f>IF(COUNT('Turns'!E31)=1,SUM('Turns'!E31),"Unknown")</f>
+        <v>0.0003295681988</v>
+      </c>
+      <c r="Z7" s="2">
+        <f>IF(COUNT('Turns'!F31)=1,SUM('Turns'!F31),"Unknown")</f>
+        <v>0.00037462</v>
+      </c>
+      <c r="AA7" s="5">
+        <f>IF(ISNUMBER(Y7),ROUND(Y7*'Reference data'!$B$2,0),"Unknown")</f>
+        <v>33.0</v>
+      </c>
+      <c r="AB7" s="5">
+        <f>IF(ISNUMBER(Z7),ROUND(Z7*'Reference data'!$B$2,0),"Unknown")</f>
+        <v>37.0</v>
       </c>
       <c r="AD7" s="1">
-        <v>1230.041</v>
+        <v>2.912</v>
       </c>
       <c r="AE7" s="1" t="s">
-        <v>130</v>
+        <v>156</v>
       </c>
     </row>
     <row r="8" spans="1:31" ht="54" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>131</v>
+        <v>160</v>
       </c>
       <c r="B8" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>124</v>
+        <v>161</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>47</v>
+        <v>126</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>111</v>
+        <v>141</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1829</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>132</v>
+        <v>162</v>
       </c>
       <c r="H8" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="I8" t="s">
-        <v>49</v>
+        <v>171</v>
       </c>
       <c r="J8" s="2">
-        <f>IF(COUNT('Turns'!D23)=1,SUM('Turns'!D23),"Unknown")</f>
-        <v>3.0</v>
+        <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
+        <v>1518.0</v>
       </c>
       <c r="K8" s="2">
-        <f>IF(COUNT('Turns'!E23)=1,SUM('Turns'!E23),"Unknown")</f>
-        <v>5.27844e-07</v>
+        <f>IF(COUNT('Turns'!E22)=1,SUM('Turns'!E22),"Unknown")</f>
+        <v>0.000267089064</v>
       </c>
       <c r="L8" s="2">
-        <f>IF(COUNT('Turns'!F23)=1,SUM('Turns'!F23),"Unknown")</f>
-        <v>6e-07</v>
+        <f>IF(COUNT('Turns'!F22)=1,SUM('Turns'!F22),"Unknown")</f>
+        <v>0.0003036</v>
       </c>
       <c r="M8" s="2">
-        <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
-        <v>2120.0</v>
+        <f>IF(COUNT('Turns'!D21)=1,SUM('Turns'!D21),"Unknown")</f>
+        <v>311.0</v>
       </c>
       <c r="N8" s="2">
-        <f>IF(COUNT('Turns'!E22)=1,SUM('Turns'!E22),"Unknown")</f>
-        <v>3.7300976e-05</v>
+        <f>IF(COUNT('Turns'!E21)=1,SUM('Turns'!E21),"Unknown")</f>
+        <v>5.4719828e-06</v>
       </c>
       <c r="O8" s="2">
-        <f>IF(COUNT('Turns'!F22)=1,SUM('Turns'!F22),"Unknown")</f>
-        <v>4.24e-05</v>
+        <f>IF(COUNT('Turns'!F21)=1,SUM('Turns'!F21),"Unknown")</f>
+        <v>6.22e-06</v>
       </c>
       <c r="P8" s="2">
-        <f>IF(COUNT('Turns'!D25)=1,SUM('Turns'!D25),"Unknown")</f>
-        <v>1507.0</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="2">
-        <f>IF(COUNT('Turns'!E25)=1,SUM('Turns'!E25),"Unknown")</f>
-        <v>0.000331442045</v>
+        <v>0</v>
       </c>
       <c r="R8" s="2">
-        <f>IF(COUNT('Turns'!F25)=1,SUM('Turns'!F25),"Unknown")</f>
-        <v>0.00037675</v>
+        <v>0</v>
       </c>
       <c r="S8" s="2">
-        <f>IF(COUNT('Turns'!D28)=1,SUM('Turns'!D28),"Unknown")</f>
-        <v>188.0</v>
+        <f>IF(COUNT('Turns'!D27)=1,SUM('Turns'!D27),"Unknown")</f>
+        <v>54.0</v>
       </c>
       <c r="T8" s="2">
-        <f>IF(COUNT('Turns'!E28)=1,SUM('Turns'!E28),"Unknown")</f>
-        <v>0.000198469344</v>
+        <f>IF(COUNT('Turns'!E27)=1,SUM('Turns'!E27),"Unknown")</f>
+        <v>5.7007152e-05</v>
       </c>
       <c r="U8" s="2">
-        <f>IF(COUNT('Turns'!F28)=1,SUM('Turns'!F28),"Unknown")</f>
-        <v>0.0002256</v>
+        <f>IF(COUNT('Turns'!F27)=1,SUM('Turns'!F27),"Unknown")</f>
+        <v>6.48e-05</v>
       </c>
       <c r="V8" s="2">
         <v>0</v>
@@ -2130,141 +2242,33 @@
         <v>0</v>
       </c>
       <c r="Y8" s="2">
-        <f>IF(COUNT('Turns'!E32)=1,SUM('Turns'!E32),"Unknown")</f>
-        <v>0.000567740209</v>
+        <f>IF(COUNT('Turns'!E31)=1,SUM('Turns'!E31),"Unknown")</f>
+        <v>0.0003295681988</v>
       </c>
       <c r="Z8" s="2">
-        <f>IF(COUNT('Turns'!F32)=1,SUM('Turns'!F32),"Unknown")</f>
-        <v>0.00064535</v>
+        <f>IF(COUNT('Turns'!F31)=1,SUM('Turns'!F31),"Unknown")</f>
+        <v>0.00037462</v>
       </c>
       <c r="AA8" s="5">
         <f>IF(ISNUMBER(Y8),ROUND(Y8*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>57.0</v>
+        <v>33.0</v>
       </c>
       <c r="AB8" s="5">
         <f>IF(ISNUMBER(Z8),ROUND(Z8*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>65.0</v>
+        <v>37.0</v>
+      </c>
+      <c r="AC8" s="1" t="s">
+        <v>148</v>
       </c>
       <c r="AD8" s="1">
-        <v>2872.138</v>
+        <v>2.069</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="9" spans="1:31" ht="54" customHeight="1">
-      <c r="A9" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="B9" s="1">
-        <v>2</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F9" s="1">
-        <v>3630</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="H9" t="s">
-        <v>119</v>
-      </c>
-      <c r="I9" t="s">
-        <v>144</v>
-      </c>
-      <c r="J9" s="2">
-        <f>IF(COUNT('Turns'!D23)=1,SUM('Turns'!D23),"Unknown")</f>
-        <v>3.0</v>
-      </c>
-      <c r="K9" s="2">
-        <f>IF(COUNT('Turns'!E23)=1,SUM('Turns'!E23),"Unknown")</f>
-        <v>5.27844e-07</v>
-      </c>
-      <c r="L9" s="2">
-        <f>IF(COUNT('Turns'!F23)=1,SUM('Turns'!F23),"Unknown")</f>
-        <v>6e-07</v>
-      </c>
-      <c r="M9" s="2">
-        <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
-        <v>2120.0</v>
-      </c>
-      <c r="N9" s="2">
-        <f>IF(COUNT('Turns'!E22)=1,SUM('Turns'!E22),"Unknown")</f>
-        <v>3.7300976e-05</v>
-      </c>
-      <c r="O9" s="2">
-        <f>IF(COUNT('Turns'!F22)=1,SUM('Turns'!F22),"Unknown")</f>
-        <v>4.24e-05</v>
-      </c>
-      <c r="P9" s="2">
-        <f>IF(COUNT('Turns'!D25)=1,SUM('Turns'!D25),"Unknown")</f>
-        <v>1507.0</v>
-      </c>
-      <c r="Q9" s="2">
-        <f>IF(COUNT('Turns'!E25)=1,SUM('Turns'!E25),"Unknown")</f>
-        <v>0.000331442045</v>
-      </c>
-      <c r="R9" s="2">
-        <f>IF(COUNT('Turns'!F25)=1,SUM('Turns'!F25),"Unknown")</f>
-        <v>0.00037675</v>
-      </c>
-      <c r="S9" s="2">
-        <f>IF(COUNT('Turns'!D28)=1,SUM('Turns'!D28),"Unknown")</f>
-        <v>188.0</v>
-      </c>
-      <c r="T9" s="2">
-        <f>IF(COUNT('Turns'!E28)=1,SUM('Turns'!E28),"Unknown")</f>
-        <v>0.000198469344</v>
-      </c>
-      <c r="U9" s="2">
-        <f>IF(COUNT('Turns'!F28)=1,SUM('Turns'!F28),"Unknown")</f>
-        <v>0.0002256</v>
-      </c>
-      <c r="V9" s="2">
-        <v>0</v>
-      </c>
-      <c r="W9" s="2">
-        <v>0</v>
-      </c>
-      <c r="X9" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y9" s="2">
-        <f>IF(COUNT('Turns'!E32)=1,SUM('Turns'!E32),"Unknown")</f>
-        <v>0.000567740209</v>
-      </c>
-      <c r="Z9" s="2">
-        <f>IF(COUNT('Turns'!F32)=1,SUM('Turns'!F32),"Unknown")</f>
-        <v>0.00064535</v>
-      </c>
-      <c r="AA9" s="5">
-        <f>IF(ISNUMBER(Y9),ROUND(Y9*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>57.0</v>
-      </c>
-      <c r="AB9" s="5">
-        <f>IF(ISNUMBER(Z9),ROUND(Z9*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>65.0</v>
-      </c>
-      <c r="AC9" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="AD9" s="1">
-        <v>2858.79</v>
-      </c>
-      <c r="AE9" s="1" t="s">
-        <v>137</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:AE9">
+  <conditionalFormatting sqref="A2:AE8">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$E2="error"</formula>
     </cfRule>
@@ -2278,7 +2282,7 @@
   <sheetPr>
     <tabColor rgb="FF173B70"/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="34.7109375" customWidth="1"/>
@@ -2663,6 +2667,731 @@
         <v>80</v>
       </c>
     </row>
+    <row r="23" spans="1:9" ht="72" customHeight="1">
+      <c r="A23" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B23" s="2">
+        <v>1</v>
+      </c>
+      <c r="C23" s="2">
+        <v>0.10</v>
+      </c>
+      <c r="D23" s="2">
+        <v>1.25</v>
+      </c>
+      <c r="E23" s="2">
+        <v>5</v>
+      </c>
+      <c r="F23" s="2">
+        <v>5</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="72" customHeight="1">
+      <c r="A24" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B24" s="2">
+        <v>1</v>
+      </c>
+      <c r="C24" s="2">
+        <v>0.10</v>
+      </c>
+      <c r="D24" s="2">
+        <v>1.25</v>
+      </c>
+      <c r="E24" s="2">
+        <v>5</v>
+      </c>
+      <c r="F24" s="2">
+        <v>5</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="72" customHeight="1">
+      <c r="A25" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B25" s="2">
+        <v>4</v>
+      </c>
+      <c r="C25" s="2">
+        <v>0.20</v>
+      </c>
+      <c r="D25" s="2">
+        <v>5</v>
+      </c>
+      <c r="E25" s="2">
+        <v>20</v>
+      </c>
+      <c r="F25" s="2">
+        <v>20</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="72" customHeight="1">
+      <c r="A26" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B26" s="2">
+        <v>3</v>
+      </c>
+      <c r="C26" s="2">
+        <v>0.30</v>
+      </c>
+      <c r="D26" s="2">
+        <v>3.75</v>
+      </c>
+      <c r="E26" s="2">
+        <v>15</v>
+      </c>
+      <c r="F26" s="2">
+        <v>15</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="72" customHeight="1">
+      <c r="A27" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B27" s="2">
+        <v>2</v>
+      </c>
+      <c r="C27" s="2">
+        <v>0.20</v>
+      </c>
+      <c r="D27" s="2">
+        <v>2.50</v>
+      </c>
+      <c r="E27" s="2">
+        <v>10</v>
+      </c>
+      <c r="F27" s="2">
+        <v>10</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="72" customHeight="1">
+      <c r="A28" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B28" s="2">
+        <v>1.00</v>
+      </c>
+      <c r="C28" s="2">
+        <v>0.10</v>
+      </c>
+      <c r="D28" s="2">
+        <v>1.25</v>
+      </c>
+      <c r="E28" s="2">
+        <v>5.00</v>
+      </c>
+      <c r="F28" s="2">
+        <v>5.00</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="72" customHeight="1">
+      <c r="A29" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B29" s="2">
+        <v>4.00</v>
+      </c>
+      <c r="C29" s="2">
+        <v>0.20</v>
+      </c>
+      <c r="D29" s="2">
+        <v>5.00</v>
+      </c>
+      <c r="E29" s="2">
+        <v>20.00</v>
+      </c>
+      <c r="F29" s="2">
+        <v>20.00</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="72" customHeight="1">
+      <c r="A30" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B30" s="2">
+        <v>3.00</v>
+      </c>
+      <c r="C30" s="2">
+        <v>0.30</v>
+      </c>
+      <c r="D30" s="2">
+        <v>3.75</v>
+      </c>
+      <c r="E30" s="2">
+        <v>15.00</v>
+      </c>
+      <c r="F30" s="2">
+        <v>15.00</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="72" customHeight="1">
+      <c r="A31" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B31" s="2">
+        <v>2.00</v>
+      </c>
+      <c r="C31" s="2">
+        <v>0.20</v>
+      </c>
+      <c r="D31" s="2">
+        <v>2.50</v>
+      </c>
+      <c r="E31" s="2">
+        <v>10.00</v>
+      </c>
+      <c r="F31" s="2">
+        <v>10.00</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="72" customHeight="1">
+      <c r="A32" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B32" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="C32" s="2">
+        <v>0.075</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E32" s="2">
+        <v>3.75</v>
+      </c>
+      <c r="F32" s="2">
+        <v>3.75</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="72" customHeight="1">
+      <c r="A33" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B33" s="2">
+        <v>1.75</v>
+      </c>
+      <c r="C33" s="2">
+        <v>0.175</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E33" s="2">
+        <v>14.00</v>
+      </c>
+      <c r="F33" s="2">
+        <v>14.00</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="72" customHeight="1">
+      <c r="A34" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34" s="2">
+        <v>2.50</v>
+      </c>
+      <c r="C34" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E34" s="2">
+        <v>15.00</v>
+      </c>
+      <c r="F34" s="2">
+        <v>15.00</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="72" customHeight="1">
+      <c r="A35" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B35" s="2">
+        <v>10.00</v>
+      </c>
+      <c r="C35" s="2">
+        <v>1.00</v>
+      </c>
+      <c r="D35" s="2">
+        <v>12.50</v>
+      </c>
+      <c r="E35" s="2">
+        <v>50.00</v>
+      </c>
+      <c r="F35" s="2">
+        <v>50.00</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="72" customHeight="1">
+      <c r="A36" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B36" s="2">
+        <v>0.10</v>
+      </c>
+      <c r="C36" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="D36" s="2">
+        <v>0.125</v>
+      </c>
+      <c r="E36" s="2">
+        <v>0.50</v>
+      </c>
+      <c r="F36" s="2">
+        <v>0.50</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="72" customHeight="1">
+      <c r="A37" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B37" s="2">
+        <v>2.00</v>
+      </c>
+      <c r="C37" s="2">
+        <v>0.20</v>
+      </c>
+      <c r="D37" s="2">
+        <v>2.50</v>
+      </c>
+      <c r="E37" s="2">
+        <v>10.00</v>
+      </c>
+      <c r="F37" s="2">
+        <v>10.00</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="72" customHeight="1">
+      <c r="A38" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B38" s="2">
+        <v>2.00</v>
+      </c>
+      <c r="C38" s="2">
+        <v>0.10</v>
+      </c>
+      <c r="D38" s="2">
+        <v>2.50</v>
+      </c>
+      <c r="E38" s="2">
+        <v>10.00</v>
+      </c>
+      <c r="F38" s="2">
+        <v>10.00</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="72" customHeight="1">
+      <c r="A39" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B39" s="2">
+        <v>10</v>
+      </c>
+      <c r="C39" s="2">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2">
+        <v>12.50</v>
+      </c>
+      <c r="E39" s="2">
+        <v>50</v>
+      </c>
+      <c r="F39" s="2">
+        <v>50</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="72" customHeight="1">
+      <c r="A40" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B40" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C40" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="D40" s="2">
+        <v>0.125</v>
+      </c>
+      <c r="E40" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F40" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="I40" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="72" customHeight="1">
+      <c r="A41" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B41" s="2">
+        <v>2</v>
+      </c>
+      <c r="C41" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D41" s="2">
+        <v>2.50</v>
+      </c>
+      <c r="E41" s="2">
+        <v>10</v>
+      </c>
+      <c r="F41" s="2">
+        <v>10</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="72" customHeight="1">
+      <c r="A42" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B42" s="2">
+        <v>2</v>
+      </c>
+      <c r="C42" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D42" s="2">
+        <v>2.50</v>
+      </c>
+      <c r="E42" s="2">
+        <v>10</v>
+      </c>
+      <c r="F42" s="2">
+        <v>10</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="I42" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="72" customHeight="1">
+      <c r="A43" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B43" s="2">
+        <v>5.00</v>
+      </c>
+      <c r="C43" s="2">
+        <v>0.50</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E43" s="2">
+        <v>22.50</v>
+      </c>
+      <c r="F43" s="2">
+        <v>22.50</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I43" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="72" customHeight="1">
+      <c r="A44" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B44" s="2">
+        <v>20.00</v>
+      </c>
+      <c r="C44" s="2">
+        <v>2.00</v>
+      </c>
+      <c r="D44" s="2">
+        <v>25.00</v>
+      </c>
+      <c r="E44" s="2">
+        <v>75.00</v>
+      </c>
+      <c r="F44" s="2">
+        <v>75.00</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="72" customHeight="1">
+      <c r="A45" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B45" s="2">
+        <v>0.20</v>
+      </c>
+      <c r="C45" s="2">
+        <v>0.02</v>
+      </c>
+      <c r="D45" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="E45" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="F45" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I45" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="72" customHeight="1">
+      <c r="A46" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B46" s="2">
+        <v>4.00</v>
+      </c>
+      <c r="C46" s="2">
+        <v>0.40</v>
+      </c>
+      <c r="D46" s="2">
+        <v>5.00</v>
+      </c>
+      <c r="E46" s="2">
+        <v>15.00</v>
+      </c>
+      <c r="F46" s="2">
+        <v>15.00</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I46" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="72" customHeight="1">
+      <c r="A47" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B47" s="2">
+        <v>4.00</v>
+      </c>
+      <c r="C47" s="2">
+        <v>0.20</v>
+      </c>
+      <c r="D47" s="2">
+        <v>5.00</v>
+      </c>
+      <c r="E47" s="2">
+        <v>15.00</v>
+      </c>
+      <c r="F47" s="2">
+        <v>15.00</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I47" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2">

</xml_diff>